<commit_message>
Plan Sushi Bar ES · F2 cerrada: los 4 entregables regenerados tras la revisión (gates verdes) y F2-NOTAS
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-sushi-bar/calculadora-pescado-arroz-escandallo-sushi-bar.xlsx
+++ b/astro-site/public/dl/plan-negocio-sushi-bar/calculadora-pescado-arroz-escandallo-sushi-bar.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Salmón noruego entero de acuicultura: unos 11,95 €/kg en minorista y 6-7,5 € en origen; lomo o filete congelado, de 20,7 a 21,8 €/kg (Makro); atún aleta amarilla en saku ultracongelado, 26 €/kg. El kit pone 9,50 · 21,80 · 26,00 €/kg. Estimación del kit, editable.</t>
+          <t>Salmón noruego entero de acuicultura: unos 11,95 €/kg en minorista y 6-7,5 € en origen; lomo o filete congelado, de 20,7 a 21,8 €/kg (Makro); el atún aleta amarilla en saku ultracongelado no tiene precio publicado en España. El kit pone 9,50 · 21,80 · 26,00 €/kg. Estimación del kit, editable.</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Entre 1,81 €/kg (METRO Chef, 5 kg) y 1,85 €/kg (DACSA, 5 kg), 2,50 € en saco de 20 kg. Estimación del kit, editable.</t>
+          <t>Entre 1,81 €/kg (METRO Chef, 5 kg) y 1,85 €/kg (DACSA, 5 kg); otra marca, a 2,50 €/kg en saco de 20 kg. Estimación del kit, editable.</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2. El coste por kilo útil es el precio ÷ (rendimiento + recorte) ÷ (1 − merma de vitrina). Es el número que alimenta el escandallo: con los valores del kit sale a 14,29 €/kg en el salmón entero, 24,15 en el lomo comprado y 28,81 en el atún en saku.</t>
+          <t>2. El coste por kilo útil es el precio ÷ (rendimiento + recorte) ÷ (1 − merma de vitrina). Es el número que alimenta el escandallo: con los valores del kit sale a 14,29 €/kg en el salmón entero, 24,16 en el lomo comprado y 28,81 en el atún en saku.</t>
         </is>
       </c>
     </row>
@@ -3469,7 +3469,7 @@
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Tu comparación real es esta: las compras de comida del mes ÷ las ventas de comida sin IVA del mes. Si después del primer trimestre sale por debajo del 29 %, cambia la celda «Coste de mercancía sobre las ventas de COMIDA» del plan: cada punto vale unos 4.000 € al año.</t>
+          <t>Tu comparación real es esta: las compras de comida del mes ÷ las ventas de comida sin IVA del mes. Si después del primer trimestre sale por encima o por debajo del 29 %, cambia la celda «Coste de mercancía sobre las ventas de COMIDA» del plan: cada punto vale unos 4.000 € al año.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan Sushi Bar ES · F3: checklist y calculadora regenerados (pH del shari en la plantilla 02 del Kit) y F3-NOTAS cerradas
Solo cambian F3!E14 del checklist y Arroz!A3 e Instrucciones!A14 de la calculadora (diff celda a celda en el VPS).
ciclo.sh TODO VERDE · autotest 580 VERDE · cifras --calc D9 VERDE con tokens idénticos · barrido 0 · LIT255 VERDE ·
restos VERDE.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-sushi-bar/calculadora-pescado-arroz-escandallo-sushi-bar.xlsx
+++ b/astro-site/public/dl/plan-negocio-sushi-bar/calculadora-pescado-arroz-escandallo-sushi-bar.xlsx
@@ -1347,7 +1347,7 @@
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>AVISO FIJO. El pH de cada tanda se registra en el Kit de Tareas Sushi Bar (hoja 03). El shari a temperatura ambiente, sólo si tu APPCC lo justifica con el pH de cada tanda y un tiempo máximo y lo demuestras a sanidad (RD 1086/2020, art. 30.5); si no, refrigerado.</t>
+          <t>AVISO FIJO. El pH de cada tanda se registra en el Kit de Tareas Sushi Bar (plantilla 02). El shari a temperatura ambiente, sólo si tu APPCC lo justifica con el pH de cada tanda y un tiempo máximo y lo demuestras a sanidad (RD 1086/2020, art. 30.5); si no, refrigerado.</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3420,7 @@
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>3. Seguridad del shari. A temperatura ambiente solo puede mantenerse si tu APPCC lo justifica y lo demuestras a sanidad (RD 1086/2020, art. 30.5); si no, se mantiene refrigerado. El pH de 4,6 o menos es el límite crítico del APPCC del Kit de Tareas Sushi Bar, no una cifra legal. El pH de cada tanda se registra en el Kit de Tareas Sushi Bar (hoja 03).</t>
+          <t>3. Seguridad del shari. A temperatura ambiente solo puede mantenerse si tu APPCC lo justifica y lo demuestras a sanidad (RD 1086/2020, art. 30.5); si no, se mantiene refrigerado. El pH de 4,6 o menos es el límite crítico del APPCC del Kit de Tareas Sushi Bar, no una cifra legal. El pH de cada tanda se registra en el Kit de Tareas Sushi Bar (plantilla 02).</t>
         </is>
       </c>
     </row>

</xml_diff>